<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (laminas_provinciales)
</commit_message>
<xml_diff>
--- a/output/laminas_provinciales/prov_i_ingr_a_2022_antofagasta.xlsx
+++ b/output/laminas_provinciales/prov_i_ingr_a_2022_antofagasta.xlsx
@@ -52,7 +52,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-28 21:33</t>
+    <t xml:space="preserve">2026-10-05 07:01</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -485,7 +485,7 @@
         <v>1271792</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1147628</v>
+        <v>1147629</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="n">
@@ -497,7 +497,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>1295900</v>
+        <v>1295901</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="n">

</xml_diff>